<commit_message>
Add Hit@10 to evaluation and Excel tracker
</commit_message>
<xml_diff>
--- a/evaluation/rag_retrieval_evaluation_tracker.xlsx
+++ b/evaluation/rag_retrieval_evaluation_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="32">
   <si>
     <t>RAG Retrieval Evaluation Tracker</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t>Hit@5</t>
+  </si>
+  <si>
+    <t>Hit@10</t>
   </si>
   <si>
     <t>MRR</t>
@@ -187,7 +190,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -209,6 +212,17 @@
     <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color indexed="11"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
       <top style="thin">
         <color indexed="11"/>
       </top>
@@ -266,6 +280,19 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top style="thin">
+        <color indexed="12"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="12"/>
       </left>
@@ -294,6 +321,19 @@
     <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color indexed="14"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="14"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
       <top style="thin">
         <color indexed="14"/>
       </top>
@@ -339,13 +379,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top style="thin">
+        <color indexed="14"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="12"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -355,20 +408,20 @@
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="4" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -376,77 +429,95 @@
     <xf numFmtId="49" fontId="4" fillId="4" borderId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="5" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="4" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="5" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="5" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="59" fontId="0" fillId="5" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="0" fillId="5" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="6" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="5" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="10" fontId="0" fillId="6" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="59" fontId="0" fillId="6" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="0" fillId="6" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="6" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="7" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="59" fontId="0" fillId="7" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="7" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="59" fontId="0" fillId="7" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="7" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="10" fontId="0" fillId="7" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="59" fontId="0" fillId="7" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="0" fillId="7" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -672,7 +743,7 @@
         <a:solidFill>
           <a:srgbClr val="FFFFFF"/>
         </a:solidFill>
-        <a:ln w="19050" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
@@ -709,10 +780,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -951,7 +1022,7 @@
     <a:lnDef>
       <a:spPr>
         <a:noFill/>
-        <a:ln w="19050" cap="flat">
+        <a:ln w="25400" cap="flat">
           <a:solidFill>
             <a:schemeClr val="accent1"/>
           </a:solidFill>
@@ -1260,10 +1331,10 @@
             </a:solidFill>
             <a:effectLst/>
             <a:uFillTx/>
-            <a:latin typeface="Calibri"/>
-            <a:ea typeface="Calibri"/>
-            <a:cs typeface="Calibri"/>
-            <a:sym typeface="Calibri"/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+            <a:sym typeface="Helvetica Neue"/>
           </a:defRPr>
         </a:defPPr>
         <a:lvl1pPr marL="0" marR="0" indent="0" algn="l" defTabSz="914400" rtl="0" fontAlgn="auto" latinLnBrk="1" hangingPunct="0">
@@ -1505,20 +1576,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="16" style="1" customWidth="1"/>
-    <col min="2" max="2" width="55.0156" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7031" style="1" customWidth="1"/>
+    <col min="2" max="2" width="55" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14.6719" style="1" customWidth="1"/>
     <col min="4" max="4" width="27" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.2266" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20.6406" style="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1719" style="1" customWidth="1"/>
+    <col min="6" max="6" width="20.6719" style="1" customWidth="1"/>
     <col min="7" max="9" width="11" style="1" customWidth="1"/>
-    <col min="10" max="10" width="10" style="1" customWidth="1"/>
-    <col min="11" max="11" width="15" style="1" customWidth="1"/>
-    <col min="12" max="12" width="13" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.85156" style="1" customWidth="1"/>
+    <col min="10" max="11" width="10" style="1" customWidth="1"/>
+    <col min="12" max="12" width="15" style="1" customWidth="1"/>
+    <col min="13" max="13" width="13" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.85156" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.2" customHeight="1">
@@ -1533,239 +1604,255 @@
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
       <c r="I1" s="4"/>
-      <c r="J1" s="4"/>
+      <c r="J1" s="3"/>
       <c r="K1" s="4"/>
       <c r="L1" s="4"/>
+      <c r="M1" s="5"/>
     </row>
     <row r="2" ht="15" customHeight="1">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
-      <c r="I2" s="6"/>
-      <c r="J2" s="6"/>
-      <c r="K2" s="6"/>
-      <c r="L2" s="5"/>
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="6"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="A3" t="s" s="7">
+      <c r="A3" t="s" s="8">
         <v>1</v>
       </c>
-      <c r="B3" t="s" s="8">
+      <c r="B3" t="s" s="9">
         <v>2</v>
       </c>
-      <c r="C3" t="s" s="7">
+      <c r="C3" t="s" s="8">
         <v>3</v>
       </c>
-      <c r="D3" t="s" s="9">
+      <c r="D3" t="s" s="10">
         <v>4</v>
       </c>
-      <c r="E3" t="s" s="9">
+      <c r="E3" t="s" s="10">
         <v>5</v>
       </c>
-      <c r="F3" t="s" s="9">
+      <c r="F3" t="s" s="10">
         <v>6</v>
       </c>
-      <c r="G3" t="s" s="9">
+      <c r="G3" t="s" s="10">
         <v>7</v>
       </c>
-      <c r="H3" t="s" s="9">
+      <c r="H3" t="s" s="10">
         <v>8</v>
       </c>
-      <c r="I3" t="s" s="9">
+      <c r="I3" t="s" s="10">
         <v>9</v>
       </c>
-      <c r="J3" t="s" s="9">
+      <c r="J3" t="s" s="10">
         <v>10</v>
       </c>
-      <c r="K3" t="s" s="9">
+      <c r="K3" t="s" s="10">
         <v>11</v>
       </c>
-      <c r="L3" t="s" s="9">
+      <c r="L3" t="s" s="10">
         <v>12</v>
+      </c>
+      <c r="M3" t="s" s="11">
+        <v>13</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" t="s" s="10">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s" s="11">
+      <c r="A4" t="s" s="12">
         <v>14</v>
       </c>
-      <c r="C4" t="s" s="10">
+      <c r="B4" t="s" s="13">
         <v>15</v>
       </c>
-      <c r="D4" t="s" s="12">
+      <c r="C4" t="s" s="12">
         <v>16</v>
       </c>
-      <c r="E4" s="13">
+      <c r="D4" t="s" s="14">
+        <v>17</v>
+      </c>
+      <c r="E4" s="15">
         <v>10</v>
       </c>
-      <c r="F4" t="s" s="12">
-        <v>17</v>
-      </c>
-      <c r="G4" s="14">
+      <c r="F4" t="s" s="14">
+        <v>18</v>
+      </c>
+      <c r="G4" s="16">
         <v>0</v>
       </c>
-      <c r="H4" s="14">
+      <c r="H4" s="16">
         <v>0</v>
       </c>
-      <c r="I4" s="14">
+      <c r="I4" s="16">
         <v>0</v>
       </c>
-      <c r="J4" s="15">
+      <c r="J4" s="16">
+        <v>0.1429</v>
+      </c>
+      <c r="K4" s="17">
         <v>0.024</v>
       </c>
-      <c r="K4" s="13">
+      <c r="L4" s="15">
         <v>7</v>
       </c>
-      <c r="L4" t="s" s="12">
-        <v>18</v>
+      <c r="M4" t="s" s="18">
+        <v>19</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
-      <c r="A5" t="s" s="16">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s" s="17">
+      <c r="A5" t="s" s="19">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s" s="20">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s" s="19">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s" s="21">
+        <v>17</v>
+      </c>
+      <c r="E5" s="22">
+        <v>10</v>
+      </c>
+      <c r="F5" t="s" s="21">
+        <v>18</v>
+      </c>
+      <c r="G5" s="23">
+        <v>0.5714</v>
+      </c>
+      <c r="H5" s="23">
+        <v>0.5714</v>
+      </c>
+      <c r="I5" s="23">
+        <v>0.5714</v>
+      </c>
+      <c r="J5" s="23">
+        <v>0.5714</v>
+      </c>
+      <c r="K5" s="24">
+        <v>0.571</v>
+      </c>
+      <c r="L5" s="22">
+        <v>7</v>
+      </c>
+      <c r="M5" t="s" s="25">
         <v>19</v>
-      </c>
-      <c r="C5" t="s" s="16">
-        <v>20</v>
-      </c>
-      <c r="D5" t="s" s="18">
-        <v>16</v>
-      </c>
-      <c r="E5" s="19">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s" s="18">
-        <v>17</v>
-      </c>
-      <c r="G5" s="20">
-        <v>0.5714</v>
-      </c>
-      <c r="H5" s="20">
-        <v>0.5714</v>
-      </c>
-      <c r="I5" s="20">
-        <v>0.5714</v>
-      </c>
-      <c r="J5" s="21">
-        <v>0.571</v>
-      </c>
-      <c r="K5" s="19">
-        <v>7</v>
-      </c>
-      <c r="L5" t="s" s="18">
-        <v>18</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
-      <c r="A6" t="s" s="10">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s" s="11">
-        <v>21</v>
-      </c>
-      <c r="C6" t="s" s="10">
+      <c r="A6" t="s" s="12">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s" s="13">
         <v>22</v>
       </c>
-      <c r="D6" t="s" s="12">
-        <v>16</v>
-      </c>
-      <c r="E6" s="13">
+      <c r="C6" t="s" s="12">
+        <v>23</v>
+      </c>
+      <c r="D6" t="s" s="14">
+        <v>17</v>
+      </c>
+      <c r="E6" s="15">
         <v>5</v>
       </c>
-      <c r="F6" t="s" s="12">
-        <v>17</v>
-      </c>
-      <c r="G6" s="14">
+      <c r="F6" t="s" s="14">
+        <v>18</v>
+      </c>
+      <c r="G6" s="16">
         <v>0</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="16">
         <v>0.1429</v>
       </c>
-      <c r="I6" s="14">
+      <c r="I6" s="16">
         <v>0.4286</v>
       </c>
-      <c r="J6" s="15">
+      <c r="J6" s="16">
+        <v>0.4286</v>
+      </c>
+      <c r="K6" s="17">
         <v>0.119</v>
       </c>
-      <c r="K6" s="13">
+      <c r="L6" s="15">
         <v>7</v>
       </c>
-      <c r="L6" t="s" s="12">
-        <v>18</v>
+      <c r="M6" t="s" s="18">
+        <v>19</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" t="s" s="22">
-        <v>23</v>
-      </c>
-      <c r="B7" t="s" s="23">
+      <c r="A7" t="s" s="26">
         <v>24</v>
       </c>
-      <c r="C7" t="s" s="22">
+      <c r="B7" t="s" s="27">
         <v>25</v>
       </c>
-      <c r="D7" t="s" s="24">
-        <v>16</v>
-      </c>
-      <c r="E7" s="25">
+      <c r="C7" t="s" s="26">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s" s="28">
+        <v>17</v>
+      </c>
+      <c r="E7" s="29">
         <v>5</v>
       </c>
-      <c r="F7" t="s" s="24">
-        <v>26</v>
-      </c>
-      <c r="G7" s="26"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="26"/>
-      <c r="J7" s="27"/>
-      <c r="K7" s="25">
+      <c r="F7" t="s" s="28">
+        <v>27</v>
+      </c>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
+      <c r="I7" s="30"/>
+      <c r="J7" s="31"/>
+      <c r="K7" s="31"/>
+      <c r="L7" s="29">
         <v>7</v>
       </c>
-      <c r="L7" t="s" s="24">
-        <v>27</v>
+      <c r="M7" t="s" s="32">
+        <v>28</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" t="s" s="28">
+      <c r="A8" t="s" s="33">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s" s="34">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s" s="33">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s" s="35">
+        <v>31</v>
+      </c>
+      <c r="E8" s="36">
+        <v>5</v>
+      </c>
+      <c r="F8" t="s" s="35">
+        <v>27</v>
+      </c>
+      <c r="G8" s="37"/>
+      <c r="H8" s="37"/>
+      <c r="I8" s="37"/>
+      <c r="J8" s="38"/>
+      <c r="K8" s="38"/>
+      <c r="L8" s="36">
+        <v>7</v>
+      </c>
+      <c r="M8" t="s" s="39">
         <v>28</v>
-      </c>
-      <c r="B8" t="s" s="29">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s" s="28">
-        <v>25</v>
-      </c>
-      <c r="D8" t="s" s="30">
-        <v>30</v>
-      </c>
-      <c r="E8" s="31">
-        <v>5</v>
-      </c>
-      <c r="F8" t="s" s="30">
-        <v>26</v>
-      </c>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="33"/>
-      <c r="K8" s="31">
-        <v>7</v>
-      </c>
-      <c r="L8" t="s" s="30">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A1:M1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>

<commit_message>
Add Docling chunking experiment, golden set, and evaluation results
</commit_message>
<xml_diff>
--- a/evaluation/rag_retrieval_evaluation_tracker.xlsx
+++ b/evaluation/rag_retrieval_evaluation_tracker.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="25">
   <si>
     <t>RAG Retrieval Evaluation Tracker</t>
   </si>
@@ -19,9 +19,6 @@
     <t>Version</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>Retrieval</t>
   </si>
   <si>
@@ -58,9 +55,6 @@
     <t>Baseline v1</t>
   </si>
   <si>
-    <t>Keyword baseline</t>
-  </si>
-  <si>
     <t>Keyword</t>
   </si>
   <si>
@@ -73,40 +67,25 @@
     <t>Completed</t>
   </si>
   <si>
-    <t>Semantic baseline</t>
-  </si>
-  <si>
     <t>Semantic</t>
   </si>
   <si>
-    <t>Hybrid baseline. Equal weight RRF</t>
-  </si>
-  <si>
     <t>Hybrid RRF</t>
   </si>
   <si>
-    <t>Improvement 1</t>
-  </si>
-  <si>
-    <t>Retrieve broader candidate set, then rerank using cross-encoder</t>
-  </si>
-  <si>
-    <t>Reranker</t>
-  </si>
-  <si>
-    <t>Cross-encoder</t>
-  </si>
-  <si>
-    <t>Planned</t>
-  </si>
-  <si>
-    <t>Improvement 2</t>
-  </si>
-  <si>
-    <t>Preserve the row and column relationships with table aware ingestion</t>
-  </si>
-  <si>
-    <t>Table aware ingestion</t>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Docling v1</t>
+  </si>
+  <si>
+    <t>Structure-aware chunking using Docling</t>
+  </si>
+  <si>
+    <t>28.57%</t>
+  </si>
+  <si>
+    <t>0.00%</t>
   </si>
 </sst>
 </file>
@@ -146,7 +125,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -189,8 +168,20 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="18"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="19"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="17">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -246,7 +237,9 @@
       <left style="thin">
         <color indexed="12"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color indexed="12"/>
+      </right>
       <top style="thin">
         <color indexed="12"/>
       </top>
@@ -256,10 +249,10 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
+      <left style="thin">
         <color indexed="12"/>
-      </right>
+      </left>
+      <right/>
       <top style="thin">
         <color indexed="12"/>
       </top>
@@ -296,7 +289,9 @@
       <left style="thin">
         <color indexed="12"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color indexed="12"/>
+      </right>
       <top style="thin">
         <color indexed="14"/>
       </top>
@@ -306,10 +301,10 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right style="thin">
+      <left style="thin">
         <color indexed="12"/>
-      </right>
+      </left>
+      <right/>
       <top style="thin">
         <color indexed="14"/>
       </top>
@@ -342,63 +337,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="12"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="14"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="12"/>
-      </right>
-      <top style="thin">
-        <color indexed="14"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="14"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="11"/>
-      </right>
-      <top style="thin">
-        <color indexed="14"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="12"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -477,6 +422,9 @@
     <xf numFmtId="49" fontId="0" fillId="6" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
@@ -489,35 +437,47 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="7" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="7" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="59" fontId="0" fillId="7" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="59" fontId="0" fillId="8" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="13" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="14" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="9" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="10" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="7" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="10" fontId="0" fillId="8" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="59" fontId="0" fillId="7" borderId="15" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="7" borderId="16" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -544,7 +504,9 @@
       <rgbColor rgb="ff729fb3"/>
       <rgbColor rgb="fff8fafc"/>
       <rgbColor rgb="ffe2f0d9"/>
-      <rgbColor rgb="fffff7e6"/>
+      <rgbColor rgb="ffe4f0da"/>
+      <rgbColor rgb="ffe4f0db"/>
+      <rgbColor rgb="fff9fafc"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -1576,20 +1538,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="16" style="1" customWidth="1"/>
-    <col min="2" max="2" width="55" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14.6719" style="1" customWidth="1"/>
-    <col min="4" max="4" width="27" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.1719" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20.6719" style="1" customWidth="1"/>
-    <col min="7" max="9" width="11" style="1" customWidth="1"/>
-    <col min="10" max="11" width="10" style="1" customWidth="1"/>
-    <col min="12" max="12" width="15" style="1" customWidth="1"/>
-    <col min="13" max="13" width="13" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.85156" style="1" customWidth="1"/>
+    <col min="1" max="1" width="16.2266" style="1" customWidth="1"/>
+    <col min="2" max="2" width="14.6719" style="1" customWidth="1"/>
+    <col min="3" max="3" width="31.8984" style="1" customWidth="1"/>
+    <col min="4" max="4" width="13.1719" style="1" customWidth="1"/>
+    <col min="5" max="5" width="20.6719" style="1" customWidth="1"/>
+    <col min="6" max="8" width="11" style="1" customWidth="1"/>
+    <col min="9" max="10" width="10" style="1" customWidth="1"/>
+    <col min="11" max="11" width="15" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.85156" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="19.2" customHeight="1">
@@ -1598,31 +1559,29 @@
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="4"/>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="4"/>
       <c r="K1" s="4"/>
-      <c r="L1" s="4"/>
-      <c r="M1" s="5"/>
+      <c r="L1" s="5"/>
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="6"/>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="6"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="7"/>
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-      <c r="M2" s="6"/>
+      <c r="L2" s="6"/>
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" t="s" s="8">
@@ -1631,7 +1590,7 @@
       <c r="B3" t="s" s="9">
         <v>2</v>
       </c>
-      <c r="C3" t="s" s="8">
+      <c r="C3" t="s" s="10">
         <v>3</v>
       </c>
       <c r="D3" t="s" s="10">
@@ -1658,31 +1617,28 @@
       <c r="K3" t="s" s="10">
         <v>11</v>
       </c>
-      <c r="L3" t="s" s="10">
+      <c r="L3" t="s" s="11">
         <v>12</v>
-      </c>
-      <c r="M3" t="s" s="11">
-        <v>13</v>
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" t="s" s="12">
+        <v>13</v>
+      </c>
+      <c r="B4" t="s" s="13">
         <v>14</v>
       </c>
-      <c r="B4" t="s" s="13">
+      <c r="C4" t="s" s="14">
         <v>15</v>
       </c>
-      <c r="C4" t="s" s="12">
+      <c r="D4" s="15">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s" s="14">
         <v>16</v>
       </c>
-      <c r="D4" t="s" s="14">
-        <v>17</v>
-      </c>
-      <c r="E4" s="15">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s" s="14">
-        <v>18</v>
+      <c r="F4" s="16">
+        <v>0</v>
       </c>
       <c r="G4" s="16">
         <v>0</v>
@@ -1691,39 +1647,36 @@
         <v>0</v>
       </c>
       <c r="I4" s="16">
-        <v>0</v>
-      </c>
-      <c r="J4" s="16">
         <v>0.1429</v>
       </c>
-      <c r="K4" s="17">
+      <c r="J4" s="17">
         <v>0.024</v>
       </c>
-      <c r="L4" s="15">
+      <c r="K4" s="15">
         <v>7</v>
       </c>
-      <c r="M4" t="s" s="18">
-        <v>19</v>
+      <c r="L4" t="s" s="18">
+        <v>17</v>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" t="s" s="19">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s" s="20">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s" s="19">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s" s="21">
-        <v>17</v>
-      </c>
-      <c r="E5" s="22">
+        <v>18</v>
+      </c>
+      <c r="C5" t="s" s="21">
+        <v>15</v>
+      </c>
+      <c r="D5" s="22">
         <v>10</v>
       </c>
-      <c r="F5" t="s" s="21">
-        <v>18</v>
+      <c r="E5" t="s" s="21">
+        <v>16</v>
+      </c>
+      <c r="F5" s="23">
+        <v>0.5714</v>
       </c>
       <c r="G5" s="23">
         <v>0.5714</v>
@@ -1734,125 +1687,171 @@
       <c r="I5" s="23">
         <v>0.5714</v>
       </c>
-      <c r="J5" s="23">
-        <v>0.5714</v>
-      </c>
-      <c r="K5" s="24">
+      <c r="J5" s="24">
         <v>0.571</v>
       </c>
-      <c r="L5" s="22">
+      <c r="K5" s="22">
         <v>7</v>
       </c>
-      <c r="M5" t="s" s="25">
-        <v>19</v>
+      <c r="L5" t="s" s="25">
+        <v>17</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" t="s" s="12">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s" s="13">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s" s="12">
-        <v>23</v>
-      </c>
-      <c r="D6" t="s" s="14">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s" s="14">
+        <v>15</v>
+      </c>
+      <c r="D6" s="15">
+        <v>5</v>
+      </c>
+      <c r="E6" t="s" s="14">
+        <v>16</v>
+      </c>
+      <c r="F6" s="16">
+        <v>0</v>
+      </c>
+      <c r="G6" s="16">
+        <v>0.1429</v>
+      </c>
+      <c r="H6" s="16">
+        <v>0.4286</v>
+      </c>
+      <c r="I6" t="s" s="26">
+        <v>20</v>
+      </c>
+      <c r="J6" s="17">
+        <v>0.119</v>
+      </c>
+      <c r="K6" s="15">
+        <v>7</v>
+      </c>
+      <c r="L6" t="s" s="18">
         <v>17</v>
-      </c>
-      <c r="E6" s="15">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s" s="14">
-        <v>18</v>
-      </c>
-      <c r="G6" s="16">
-        <v>0</v>
-      </c>
-      <c r="H6" s="16">
-        <v>0.1429</v>
-      </c>
-      <c r="I6" s="16">
-        <v>0.4286</v>
-      </c>
-      <c r="J6" s="16">
-        <v>0.4286</v>
-      </c>
-      <c r="K6" s="17">
-        <v>0.119</v>
-      </c>
-      <c r="L6" s="15">
-        <v>7</v>
-      </c>
-      <c r="M6" t="s" s="18">
-        <v>19</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
-      <c r="A7" t="s" s="26">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s" s="27">
-        <v>25</v>
-      </c>
-      <c r="C7" t="s" s="26">
-        <v>26</v>
-      </c>
-      <c r="D7" t="s" s="28">
+      <c r="A7" t="s" s="27">
+        <v>21</v>
+      </c>
+      <c r="B7" t="s" s="28">
+        <v>14</v>
+      </c>
+      <c r="C7" t="s" s="29">
+        <v>22</v>
+      </c>
+      <c r="D7" s="30">
+        <v>10</v>
+      </c>
+      <c r="E7" t="s" s="29">
+        <v>16</v>
+      </c>
+      <c r="F7" t="s" s="31">
+        <v>23</v>
+      </c>
+      <c r="G7" t="s" s="31">
+        <v>23</v>
+      </c>
+      <c r="H7" t="s" s="31">
+        <v>23</v>
+      </c>
+      <c r="I7" t="s" s="31">
+        <v>23</v>
+      </c>
+      <c r="J7" s="32">
+        <v>0.286</v>
+      </c>
+      <c r="K7" s="30">
+        <v>7</v>
+      </c>
+      <c r="L7" t="s" s="25">
         <v>17</v>
-      </c>
-      <c r="E7" s="29">
-        <v>5</v>
-      </c>
-      <c r="F7" t="s" s="28">
-        <v>27</v>
-      </c>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-      <c r="I7" s="30"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="31"/>
-      <c r="L7" s="29">
-        <v>7</v>
-      </c>
-      <c r="M7" t="s" s="32">
-        <v>28</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" t="s" s="33">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B8" t="s" s="34">
-        <v>30</v>
-      </c>
-      <c r="C8" t="s" s="33">
-        <v>26</v>
-      </c>
-      <c r="D8" t="s" s="35">
-        <v>31</v>
-      </c>
-      <c r="E8" s="36">
+        <v>18</v>
+      </c>
+      <c r="C8" t="s" s="35">
+        <v>22</v>
+      </c>
+      <c r="D8" s="36">
+        <v>10</v>
+      </c>
+      <c r="E8" t="s" s="35">
+        <v>16</v>
+      </c>
+      <c r="F8" s="37">
+        <v>0</v>
+      </c>
+      <c r="G8" t="s" s="38">
+        <v>24</v>
+      </c>
+      <c r="H8" t="s" s="38">
+        <v>24</v>
+      </c>
+      <c r="I8" t="s" s="26">
+        <v>23</v>
+      </c>
+      <c r="J8" s="17">
+        <v>0.04</v>
+      </c>
+      <c r="K8" s="36">
+        <v>7</v>
+      </c>
+      <c r="L8" t="s" s="18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" t="s" s="39">
+        <v>21</v>
+      </c>
+      <c r="B9" t="s" s="40">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s" s="41">
+        <v>22</v>
+      </c>
+      <c r="D9" s="42">
         <v>5</v>
       </c>
-      <c r="F8" t="s" s="35">
-        <v>27</v>
-      </c>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="37"/>
-      <c r="J8" s="38"/>
-      <c r="K8" s="38"/>
-      <c r="L8" s="36">
+      <c r="E9" t="s" s="41">
+        <v>16</v>
+      </c>
+      <c r="F9" s="43">
+        <v>0</v>
+      </c>
+      <c r="G9" t="s" s="44">
+        <v>23</v>
+      </c>
+      <c r="H9" t="s" s="44">
+        <v>23</v>
+      </c>
+      <c r="I9" t="s" s="44">
+        <v>20</v>
+      </c>
+      <c r="J9" s="32">
+        <v>0.119</v>
+      </c>
+      <c r="K9" s="42">
         <v>7</v>
       </c>
-      <c r="M8" t="s" s="39">
-        <v>28</v>
+      <c r="L9" t="s" s="25">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup firstPageNumber="1" fitToHeight="1" fitToWidth="1" scale="100" useFirstPageNumber="0" orientation="portrait" pageOrder="downThenOver"/>

</xml_diff>